<commit_message>
Fix: linter issues, remade README, configs
</commit_message>
<xml_diff>
--- a/data/processed/summary_table1.xlsx
+++ b/data/processed/summary_table1.xlsx
@@ -34,7 +34,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="44">
+  <fills count="40">
     <fill>
       <patternFill/>
     </fill>
@@ -68,47 +68,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E55D5C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E67371"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0EEEB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="007A98BD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E5E7E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E77C7A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1D8DF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="008DA6C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E88785"/>
+        <fgColor rgb="00EAA19F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAA8A6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E99A98"/>
       </patternFill>
     </fill>
     <fill>
@@ -118,52 +88,102 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E3E5E7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E6706E"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EED5D2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E88B89"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E88E8C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A8BACF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DFE2E5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EED7D4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E78280"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EFDCD9"/>
+        <fgColor rgb="00EFE0DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDCBC8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C4CEDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBB4B1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBB4B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBB0AD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E34948"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECBBB9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CAD3DD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D7DDE2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CFD7DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0EBE8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00AABBD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E9E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEDBD9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1D8E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDC9D7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6E7E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECBAB8"/>
       </patternFill>
     </fill>
     <fill>
@@ -173,42 +193,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EED3D0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E9EAE9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EED8D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DADEE3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1D8E0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDEDEB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D2D9E0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EFDDDA"/>
+        <fgColor rgb="00EFDEDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0090A8C5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0091A8C6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006C8DB7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006185B2"/>
       </patternFill>
     </fill>
     <fill>
@@ -218,37 +223,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="007D9ABE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F0EAE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00A1B5CC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D4DAE1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00ACBDD1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BFCBD8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EED9D6"/>
+        <fgColor rgb="00C5CFDB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EED0CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -264,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -286,40 +266,36 @@
     <xf numFmtId="4" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="17" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="18" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="25" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="26" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="27" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="28" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="29" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="30" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="31" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="32" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="33" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="34" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="35" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="36" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="37" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="38" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="39" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="40" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="41" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="42" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="43" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -697,7 +673,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Характерные признаки кластеров, 2024 г. (ward_kmeans, k = 5, pooled; денежные — в ценах 2023 г.)</t>
+          <t>Характерные признаки кластеров, 2024 г. (ward_kmeans, k = 5, pooled; денежные — в ценах 2020 г.)</t>
         </is>
       </c>
     </row>
@@ -730,16 +706,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>157</v>
+        <v>259</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Максимальные значения: ВМП на душу населения, инвестиции на жителя без бюджетных средств, среднемесячная зарплата. Низкие значения: доля населения старше трудоспособного возраста. Минимальные значения: плотность населения.</t>
+          <t>Максимальные значения: отгрузка на жителя, инвестиции на жителя без бюджетных средств. Высокие значения: ВМП на душу населения, среднемесячная зарплата.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Альметьевский, Норильск, Березники, Сургутский</t>
+          <t>Краснодар, Воронеж, Волгоград, Томск</t>
         </is>
       </c>
     </row>
@@ -750,16 +726,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Максимальные значения: плотность населения, оборот розничной торговли на жителя. Высокие значения: ВМП на душу населения, среднемесячная зарплата, инвестиции на жителя без бюджетных средств.</t>
+          <t>Максимальные значения: бюджетная самостоятельность. Высокие значения: отгрузка на жителя, инвестиции на жителя без бюджетных средств, ВМП на душу населения, среднемесячная зарплата.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Екатеринбург, Казань, Краснодар, Нижний Новгород</t>
+          <t>Екатеринбург, Казань, Нижний Новгород, Красноярск</t>
         </is>
       </c>
     </row>
@@ -770,16 +746,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>237</v>
+        <v>582</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Высокие значения: плотность населения. Близкие к среднему: оборот розничной торговли на жителя, доля населения старше трудоспособного возраста.</t>
+          <t>Близкие к среднему: среднемесячная зарплата, доля населения старше трудоспособного возраста. Низкие значения: бюджетная самостоятельность.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Воронеж, Волгоград, Саратов, Барнаул</t>
+          <t>Копейский, Тюменский, Шалинский, Камышин</t>
         </is>
       </c>
     </row>
@@ -790,16 +766,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>954</v>
+        <v>337</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Близкие к среднему: плотность населения, среднемесячная зарплата, инвестиции на жителя без бюджетных средств.</t>
+          <t>Высокие значения: бюджетная самостоятельность. Близкие к среднему: среднемесячная зарплата, ВМП на душу населения.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Всеволожский, Сочи, Якутск, Нижний Тагил</t>
+          <t>Ставрополь, Энгельсский, Орёл, Нальчик</t>
         </is>
       </c>
     </row>
@@ -810,16 +786,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>593</v>
+        <v>344</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Низкие значения: плотность населения, ВМП на душу населения, среднемесячная зарплата. Минимальные значения: инвестиции на жителя без бюджетных средств.</t>
+          <t>Низкие значения: ВМП на душу населения, среднемесячная зарплата, бюджетная самостоятельность. Минимальные значения: отгрузка на жителя, инвестиции на жителя без бюджетных средств.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Иркутский, Хабаровский, Чегемский, Сакский</t>
+          <t>Сакский, Надтеречный, Джанкойский, Наурский</t>
         </is>
       </c>
     </row>
@@ -834,7 +810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -845,13 +821,12 @@
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Характерные признаки кластеров, 2024 г. (ward_kmeans, k = 5, pooled; денежные — в ценах 2023 г.): средние значения признаков (цвет — средний z-score: синий — ниже, красный — выше)</t>
+          <t>Характерные признаки кластеров, 2024 г. (ward_kmeans, k = 5, pooled; денежные — в ценах 2020 г.): средние значения признаков (цвет — средний z-score: синий — ниже, красный — выше)</t>
         </is>
       </c>
     </row>
@@ -868,35 +843,30 @@
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
+          <t>среднемесячная зарплата</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
           <t>инвестиции на жителя без бюджетных средств</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
-        <is>
-          <t>индекс Херфиндаля структуры занятости</t>
-        </is>
-      </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>плотность населения</t>
+          <t>отгрузка на жителя</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>темп изменения населения за год</t>
+          <t>бюджетная самостоятельность</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>среднемесячная зарплата</t>
+          <t>оборот розничной торговли на жителя</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
-        <is>
-          <t>оборот розничной торговли на жителя</t>
-        </is>
-      </c>
-      <c r="I2" s="8" t="inlineStr">
         <is>
           <t>доля населения старше трудоспособного возраста</t>
         </is>
@@ -909,152 +879,137 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>7794814.528662294</v>
+        <v>1888923.149940389</v>
       </c>
       <c r="C3" s="11" t="n">
-        <v>1993550.295575183</v>
+        <v>64739.40167611087</v>
       </c>
       <c r="D3" s="12" t="n">
-        <v>0.1765080461026665</v>
+        <v>666674.7985325735</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>3.419959240826713</v>
+        <v>2261392.176279528</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>-0.009762900294744708</v>
+        <v>36.47822393822394</v>
       </c>
       <c r="G3" s="15" t="n">
-        <v>114448.9770146997</v>
+        <v>116671.464346201</v>
       </c>
       <c r="H3" s="16" t="n">
-        <v>89296.73816074549</v>
-      </c>
-      <c r="I3" s="17" t="n">
-        <v>0.2030616887546518</v>
+        <v>0.2330730858753515</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="18" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>K2</t>
         </is>
       </c>
-      <c r="B4" s="19" t="n">
-        <v>3067750.598556687</v>
-      </c>
-      <c r="C4" s="20" t="n">
-        <v>352745.2595848565</v>
-      </c>
-      <c r="D4" s="21" t="n">
-        <v>0.1651379417657841</v>
-      </c>
-      <c r="E4" s="22" t="n">
-        <v>3777.667361342216</v>
-      </c>
-      <c r="F4" s="23" t="n">
-        <v>-0.0002455171084551751</v>
-      </c>
-      <c r="G4" s="24" t="n">
-        <v>105515.4934324359</v>
-      </c>
-      <c r="H4" s="25" t="n">
-        <v>369987.0582971504</v>
-      </c>
-      <c r="I4" s="26" t="n">
-        <v>0.2169613871876273</v>
+      <c r="B4" s="18" t="n">
+        <v>1952111.571895918</v>
+      </c>
+      <c r="C4" s="19" t="n">
+        <v>62624.24233453432</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>354314.3962783634</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>2193726.961141559</v>
+      </c>
+      <c r="F4" s="21" t="n">
+        <v>69.86568047337278</v>
+      </c>
+      <c r="G4" s="22" t="n">
+        <v>138755.8987156867</v>
+      </c>
+      <c r="H4" s="23" t="n">
+        <v>0.2361461930245273</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="24" t="inlineStr">
         <is>
           <t>K3</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
-        <v>522380.6807038709</v>
-      </c>
-      <c r="C5" s="28" t="n">
-        <v>36230.5810480022</v>
-      </c>
-      <c r="D5" s="29" t="n">
-        <v>0.1984131618002906</v>
-      </c>
-      <c r="E5" s="30" t="n">
-        <v>2616.993410453844</v>
-      </c>
-      <c r="F5" s="31" t="n">
-        <v>-0.002369122863399098</v>
-      </c>
-      <c r="G5" s="32" t="n">
-        <v>65002.24855066498</v>
-      </c>
-      <c r="H5" s="33" t="n">
-        <v>146004.6473443546</v>
-      </c>
-      <c r="I5" s="16" t="n">
-        <v>0.2382251957365376</v>
+      <c r="B5" s="25" t="n">
+        <v>297670.2624252417</v>
+      </c>
+      <c r="C5" s="26" t="n">
+        <v>44029.37184166743</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>36823.69032410632</v>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>207963.7613063923</v>
+      </c>
+      <c r="F5" s="29" t="n">
+        <v>22.04209621993127</v>
+      </c>
+      <c r="G5" s="30" t="n">
+        <v>73368.03623844396</v>
+      </c>
+      <c r="H5" s="31" t="n">
+        <v>0.2687097493116511</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="34" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t>K4</t>
         </is>
       </c>
-      <c r="B6" s="35" t="n">
-        <v>547927.2433595647</v>
-      </c>
-      <c r="C6" s="36" t="n">
-        <v>71665.66746288066</v>
-      </c>
-      <c r="D6" s="37" t="n">
-        <v>0.1583400416270406</v>
-      </c>
-      <c r="E6" s="38" t="n">
-        <v>24.50683023786105</v>
-      </c>
-      <c r="F6" s="39" t="n">
-        <v>-0.008061996435025833</v>
-      </c>
-      <c r="G6" s="40" t="n">
-        <v>56098.66818021848</v>
-      </c>
-      <c r="H6" s="39" t="n">
-        <v>101176.2560719975</v>
-      </c>
-      <c r="I6" s="41" t="n">
-        <v>0.2664890472906951</v>
+      <c r="B6" s="33" t="n">
+        <v>280229.9172002234</v>
+      </c>
+      <c r="C6" s="34" t="n">
+        <v>41800.26537415444</v>
+      </c>
+      <c r="D6" s="35" t="n">
+        <v>26224.6580953457</v>
+      </c>
+      <c r="E6" s="35" t="n">
+        <v>210972.35435153</v>
+      </c>
+      <c r="F6" s="36" t="n">
+        <v>44.3433234421365</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <v>81952.29980222814</v>
+      </c>
+      <c r="H6" s="38" t="n">
+        <v>0.2671275229321487</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="42" t="inlineStr">
+      <c r="A7" s="39" t="inlineStr">
         <is>
           <t>K5</t>
         </is>
       </c>
-      <c r="B7" s="43" t="n">
-        <v>274334.9075487445</v>
-      </c>
-      <c r="C7" s="44" t="n">
-        <v>6604.56779968723</v>
-      </c>
-      <c r="D7" s="45" t="n">
-        <v>0.1797858873484174</v>
-      </c>
-      <c r="E7" s="46" t="n">
-        <v>7.474059967920154</v>
-      </c>
-      <c r="F7" s="47" t="n">
-        <v>-0.01346305867678189</v>
-      </c>
-      <c r="G7" s="48" t="n">
-        <v>49061.06575897902</v>
-      </c>
-      <c r="H7" s="49" t="n">
-        <v>68762.94790036463</v>
-      </c>
-      <c r="I7" s="50" t="n">
-        <v>0.269466001789758</v>
+      <c r="B7" s="40" t="n">
+        <v>143987.3209858862</v>
+      </c>
+      <c r="C7" s="41" t="n">
+        <v>36575.69432954031</v>
+      </c>
+      <c r="D7" s="42" t="n">
+        <v>3806.014160415493</v>
+      </c>
+      <c r="E7" s="43" t="n">
+        <v>26535.47129513867</v>
+      </c>
+      <c r="F7" s="44" t="n">
+        <v>20.90813953488372</v>
+      </c>
+      <c r="G7" s="45" t="n">
+        <v>56080.36645363664</v>
+      </c>
+      <c r="H7" s="46" t="n">
+        <v>0.2761956420645731</v>
       </c>
     </row>
   </sheetData>

</xml_diff>